<commit_message>
update tìm kiếm PO  theo tên NCC
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/po_template.xlsx
+++ b/MPR_Managerment/Templates/po_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c02630c4a1efac79/Working/Backup/Revise_PO_WindowForm/Revise_PO_Form/Revise_PO_Form/bin/Debug/Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final\MPR_Managerment\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{F4DDEF6F-5AB0-4C2E-B448-CFEF80A7A692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8271F43F-93DC-40CE-9834-D2B639AD43DE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B003892F-78A9-418B-B493-C844ABD53D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{08BC6B50-49E0-41CF-A464-82D4FBAF0A1C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{08BC6B50-49E0-41CF-A464-82D4FBAF0A1C}"/>
   </bookViews>
   <sheets>
     <sheet name="DV-DPCII-PC-9" sheetId="1" r:id="rId1"/>
@@ -1362,10 +1362,21 @@
     <definedName name="ㅛㅛㅛ" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="実行" hidden="1">{"'Sheet1'!$L$16"}</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1865,7 +1876,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1933,11 +1944,137 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1945,27 +2082,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2020,124 +2145,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3077,40 +3085,40 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q17"/>
-  <sheetFormatPr defaultColWidth="9.88671875" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.109375" style="2" customWidth="1"/>
-    <col min="4" max="6" width="13.109375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="12.44140625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="28.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5546875" style="2" customWidth="1"/>
-    <col min="12" max="13" width="15.44140625" style="2" customWidth="1"/>
-    <col min="14" max="15" width="18.5546875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="15.44140625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="15.44140625" style="18" customWidth="1"/>
-    <col min="18" max="16384" width="9.88671875" style="2"/>
+    <col min="1" max="1" width="5.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="2" customWidth="1"/>
+    <col min="4" max="6" width="13.140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="12.42578125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="28.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" style="2" customWidth="1"/>
+    <col min="12" max="13" width="15.42578125" style="2" customWidth="1"/>
+    <col min="14" max="15" width="18.5703125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="15.42578125" style="2" customWidth="1"/>
+    <col min="17" max="17" width="15.42578125" style="18" customWidth="1"/>
+    <col min="18" max="16384" width="9.85546875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="40.5" customHeight="1">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="63" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="64"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="68"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="44"/>
       <c r="L1" s="1" t="s">
         <v>1</v>
       </c>
@@ -3131,166 +3139,166 @@
       </c>
     </row>
     <row r="2" spans="1:17" ht="40.5" customHeight="1">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="72" t="s">
+      <c r="B2" s="32"/>
+      <c r="C2" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="73"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="59" t="s">
+      <c r="D2" s="49"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="M2" s="86" t="s">
+      <c r="M2" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="N2" s="87" t="s">
+      <c r="N2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="59"/>
-      <c r="P2" s="88"/>
-      <c r="Q2" s="59"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="28"/>
+      <c r="Q2" s="27"/>
     </row>
-    <row r="3" spans="1:17" ht="22.65" customHeight="1">
-      <c r="A3" s="75" t="s">
+    <row r="3" spans="1:17" ht="22.7" customHeight="1">
+      <c r="A3" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="75"/>
-      <c r="C3" s="76" t="s">
+      <c r="B3" s="51"/>
+      <c r="C3" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="77"/>
-      <c r="E3" s="78"/>
-      <c r="F3" s="79" t="s">
+      <c r="D3" s="53"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="86"/>
-      <c r="N3" s="87"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="89"/>
-      <c r="Q3" s="59"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="25"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="27"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="27"/>
     </row>
-    <row r="4" spans="1:17" ht="22.65" customHeight="1">
-      <c r="A4" s="75"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="81" t="s">
+    <row r="4" spans="1:17" ht="22.7" customHeight="1">
+      <c r="A4" s="51"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="59" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="82"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="80"/>
-      <c r="G4" s="80"/>
-      <c r="H4" s="80"/>
-      <c r="I4" s="80"/>
-      <c r="J4" s="80"/>
-      <c r="K4" s="29"/>
-      <c r="L4" s="59"/>
-      <c r="M4" s="86"/>
-      <c r="N4" s="87"/>
-      <c r="O4" s="59"/>
-      <c r="P4" s="90"/>
-      <c r="Q4" s="59"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="25"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="30"/>
+      <c r="Q4" s="27"/>
     </row>
     <row r="5" spans="1:17" ht="66" customHeight="1">
-      <c r="A5" s="55" t="s">
+      <c r="A5" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="55"/>
-      <c r="C5" s="56" t="s">
+      <c r="B5" s="32"/>
+      <c r="C5" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="57"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="55" t="s">
+      <c r="D5" s="34"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="59"/>
-      <c r="H5" s="60" t="s">
+      <c r="G5" s="27"/>
+      <c r="H5" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="I5" s="61"/>
-      <c r="J5" s="62"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="38"/>
       <c r="K5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="91" t="s">
+      <c r="L5" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="M5" s="85"/>
+      <c r="M5" s="24"/>
       <c r="N5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="84" t="s">
+      <c r="O5" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="P5" s="85"/>
-      <c r="Q5" s="85"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="24"/>
     </row>
     <row r="6" spans="1:17" ht="18.600000000000001" customHeight="1">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="52" t="s">
+      <c r="B6" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="54"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="52" t="s">
+      <c r="E6" s="65"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="52" t="s">
+      <c r="H6" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="52" t="s">
+      <c r="I6" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="J6" s="52" t="s">
+      <c r="J6" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="52" t="s">
+      <c r="K6" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="52" t="s">
+      <c r="L6" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="M6" s="52" t="s">
+      <c r="M6" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="N6" s="52" t="s">
+      <c r="N6" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="O6" s="52" t="s">
+      <c r="O6" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="P6" s="26" t="s">
+      <c r="P6" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="Q6" s="27"/>
+      <c r="Q6" s="56"/>
     </row>
     <row r="7" spans="1:17" ht="21.6" customHeight="1">
-      <c r="A7" s="53"/>
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
+      <c r="A7" s="63"/>
+      <c r="B7" s="63"/>
+      <c r="C7" s="63"/>
       <c r="D7" s="1" t="s">
         <v>29</v>
       </c>
@@ -3300,21 +3308,21 @@
       <c r="F7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="53"/>
-      <c r="K7" s="53"/>
-      <c r="L7" s="53"/>
-      <c r="M7" s="53"/>
-      <c r="N7" s="53"/>
-      <c r="O7" s="53"/>
-      <c r="P7" s="28"/>
-      <c r="Q7" s="29"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
+      <c r="J7" s="63"/>
+      <c r="K7" s="63"/>
+      <c r="L7" s="63"/>
+      <c r="M7" s="63"/>
+      <c r="N7" s="63"/>
+      <c r="O7" s="63"/>
+      <c r="P7" s="69"/>
+      <c r="Q7" s="58"/>
     </row>
-    <row r="8" spans="1:17" ht="16.8" customHeight="1">
+    <row r="8" spans="1:17" ht="16.899999999999999" customHeight="1">
       <c r="A8" s="21"/>
-      <c r="B8" s="23"/>
+      <c r="B8" s="21"/>
       <c r="C8" s="21"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -3325,21 +3333,21 @@
       <c r="J8" s="21"/>
       <c r="K8" s="21"/>
       <c r="L8" s="21"/>
-      <c r="M8" s="24"/>
-      <c r="N8" s="24"/>
+      <c r="M8" s="90"/>
+      <c r="N8" s="90"/>
       <c r="O8" s="21"/>
       <c r="P8" s="22"/>
       <c r="Q8" s="19"/>
     </row>
-    <row r="9" spans="1:17" ht="24.9" customHeight="1">
+    <row r="9" spans="1:17" ht="24.95" customHeight="1">
       <c r="A9" s="4"/>
       <c r="B9" s="5"/>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="70" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="31"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="71"/>
       <c r="G9" s="6"/>
       <c r="H9" s="7"/>
       <c r="I9" s="6">
@@ -3354,18 +3362,18 @@
         <v>0</v>
       </c>
       <c r="O9" s="11"/>
-      <c r="P9" s="32"/>
-      <c r="Q9" s="33"/>
+      <c r="P9" s="64"/>
+      <c r="Q9" s="66"/>
     </row>
-    <row r="10" spans="1:17" ht="24.9" customHeight="1">
+    <row r="10" spans="1:17" ht="24.95" customHeight="1">
       <c r="A10" s="12"/>
       <c r="B10" s="13"/>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="72" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="35"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="72"/>
+      <c r="F10" s="73"/>
       <c r="G10" s="6"/>
       <c r="H10" s="3"/>
       <c r="I10" s="6"/>
@@ -3375,182 +3383,152 @@
       <c r="M10" s="3"/>
       <c r="N10" s="14"/>
       <c r="O10" s="15"/>
-      <c r="P10" s="32"/>
-      <c r="Q10" s="33"/>
+      <c r="P10" s="64"/>
+      <c r="Q10" s="66"/>
     </row>
     <row r="11" spans="1:17" ht="27" customHeight="1">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="37"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37"/>
-      <c r="K11" s="42" t="s">
+      <c r="B11" s="75"/>
+      <c r="C11" s="75"/>
+      <c r="D11" s="75"/>
+      <c r="E11" s="75"/>
+      <c r="F11" s="75"/>
+      <c r="G11" s="75"/>
+      <c r="H11" s="75"/>
+      <c r="I11" s="75"/>
+      <c r="J11" s="75"/>
+      <c r="K11" s="80" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="42"/>
-      <c r="M11" s="42"/>
-      <c r="N11" s="42"/>
-      <c r="O11" s="42"/>
-      <c r="P11" s="42"/>
-      <c r="Q11" s="43"/>
+      <c r="L11" s="80"/>
+      <c r="M11" s="80"/>
+      <c r="N11" s="80"/>
+      <c r="O11" s="80"/>
+      <c r="P11" s="80"/>
+      <c r="Q11" s="81"/>
     </row>
     <row r="12" spans="1:17" ht="27" customHeight="1">
-      <c r="A12" s="38"/>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="44"/>
-      <c r="L12" s="44"/>
-      <c r="M12" s="44"/>
-      <c r="N12" s="44"/>
-      <c r="O12" s="44"/>
-      <c r="P12" s="44"/>
-      <c r="Q12" s="45"/>
+      <c r="A12" s="76"/>
+      <c r="B12" s="77"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="77"/>
+      <c r="E12" s="77"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
+      <c r="I12" s="77"/>
+      <c r="J12" s="77"/>
+      <c r="K12" s="82"/>
+      <c r="L12" s="82"/>
+      <c r="M12" s="82"/>
+      <c r="N12" s="82"/>
+      <c r="O12" s="82"/>
+      <c r="P12" s="82"/>
+      <c r="Q12" s="83"/>
     </row>
     <row r="13" spans="1:17" ht="27" customHeight="1">
-      <c r="A13" s="38"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="39"/>
-      <c r="I13" s="39"/>
-      <c r="J13" s="39"/>
-      <c r="K13" s="46"/>
-      <c r="L13" s="46"/>
-      <c r="M13" s="46"/>
-      <c r="N13" s="47" t="s">
+      <c r="A13" s="76"/>
+      <c r="B13" s="77"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="77"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="77"/>
+      <c r="I13" s="77"/>
+      <c r="J13" s="77"/>
+      <c r="K13" s="84"/>
+      <c r="L13" s="84"/>
+      <c r="M13" s="84"/>
+      <c r="N13" s="85" t="s">
         <v>44</v>
       </c>
-      <c r="O13" s="48"/>
-      <c r="P13" s="48"/>
-      <c r="Q13" s="49"/>
+      <c r="O13" s="86"/>
+      <c r="P13" s="86"/>
+      <c r="Q13" s="87"/>
     </row>
     <row r="14" spans="1:17" ht="27" customHeight="1">
-      <c r="A14" s="38"/>
-      <c r="B14" s="39"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="39"/>
-      <c r="J14" s="39"/>
-      <c r="K14" s="48" t="s">
+      <c r="A14" s="76"/>
+      <c r="B14" s="77"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="77"/>
+      <c r="K14" s="86" t="s">
         <v>35</v>
       </c>
-      <c r="L14" s="48"/>
-      <c r="M14" s="48"/>
-      <c r="N14" s="48"/>
-      <c r="O14" s="48"/>
-      <c r="P14" s="48"/>
-      <c r="Q14" s="49"/>
+      <c r="L14" s="86"/>
+      <c r="M14" s="86"/>
+      <c r="N14" s="86"/>
+      <c r="O14" s="86"/>
+      <c r="P14" s="86"/>
+      <c r="Q14" s="87"/>
     </row>
     <row r="15" spans="1:17" ht="255" customHeight="1">
-      <c r="A15" s="40"/>
-      <c r="B15" s="41"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="41"/>
-      <c r="K15" s="50"/>
-      <c r="L15" s="50"/>
-      <c r="M15" s="50"/>
-      <c r="N15" s="50"/>
-      <c r="O15" s="50"/>
-      <c r="P15" s="50"/>
-      <c r="Q15" s="51"/>
+      <c r="A15" s="78"/>
+      <c r="B15" s="79"/>
+      <c r="C15" s="79"/>
+      <c r="D15" s="79"/>
+      <c r="E15" s="79"/>
+      <c r="F15" s="79"/>
+      <c r="G15" s="79"/>
+      <c r="H15" s="79"/>
+      <c r="I15" s="79"/>
+      <c r="J15" s="79"/>
+      <c r="K15" s="88"/>
+      <c r="L15" s="88"/>
+      <c r="M15" s="88"/>
+      <c r="N15" s="88"/>
+      <c r="O15" s="88"/>
+      <c r="P15" s="88"/>
+      <c r="Q15" s="89"/>
     </row>
     <row r="16" spans="1:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="A16" s="25"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
+      <c r="A16" s="67"/>
+      <c r="B16" s="67"/>
+      <c r="C16" s="67"/>
+      <c r="D16" s="67"/>
       <c r="E16" s="16"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
-      <c r="L16" s="25"/>
-      <c r="M16" s="25"/>
-      <c r="N16" s="25"/>
-      <c r="O16" s="25"/>
-      <c r="P16" s="25"/>
-      <c r="Q16" s="25"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="67"/>
+      <c r="H16" s="67"/>
+      <c r="I16" s="67"/>
+      <c r="J16" s="67"/>
+      <c r="K16" s="67"/>
+      <c r="L16" s="67"/>
+      <c r="M16" s="67"/>
+      <c r="N16" s="67"/>
+      <c r="O16" s="67"/>
+      <c r="P16" s="67"/>
+      <c r="Q16" s="67"/>
     </row>
     <row r="17" spans="1:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="A17" s="25"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
+      <c r="A17" s="67"/>
+      <c r="B17" s="67"/>
+      <c r="C17" s="67"/>
+      <c r="D17" s="67"/>
       <c r="E17" s="16"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="25"/>
-      <c r="N17" s="25"/>
-      <c r="O17" s="25"/>
-      <c r="P17" s="25"/>
-      <c r="Q17" s="25"/>
+      <c r="F17" s="67"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="67"/>
+      <c r="I17" s="67"/>
+      <c r="J17" s="67"/>
+      <c r="K17" s="67"/>
+      <c r="L17" s="67"/>
+      <c r="M17" s="67"/>
+      <c r="N17" s="67"/>
+      <c r="O17" s="67"/>
+      <c r="P17" s="67"/>
+      <c r="Q17" s="67"/>
     </row>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="M2:M4"/>
-    <mergeCell ref="N2:N4"/>
-    <mergeCell ref="O2:O4"/>
-    <mergeCell ref="P2:P4"/>
-    <mergeCell ref="Q2:Q4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L2:L4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:K2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A3:B4"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="F3:K4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="O6:O7"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="G6:G7"/>
     <mergeCell ref="A16:D17"/>
     <mergeCell ref="F16:Q17"/>
     <mergeCell ref="P6:Q7"/>
@@ -3567,9 +3545,39 @@
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="L6:L7"/>
     <mergeCell ref="M6:M7"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="F1:K2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="A3:B4"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F3:K4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="M2:M4"/>
+    <mergeCell ref="N2:N4"/>
+    <mergeCell ref="O2:O4"/>
+    <mergeCell ref="P2:P4"/>
+    <mergeCell ref="Q2:Q4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L2:L4"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="50" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="49" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix export to excel PO
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/po_template.xlsx
+++ b/MPR_Managerment/Templates/po_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final\MPR_Managerment\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Management\MPR_Managerment\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B003892F-78A9-418B-B493-C844ABD53D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1A27078-9774-469B-9590-9894E520C940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{08BC6B50-49E0-41CF-A464-82D4FBAF0A1C}"/>
   </bookViews>
@@ -139,13 +139,13 @@
     <definedName name="_Key1" hidden="1">#REF!</definedName>
     <definedName name="_Key2" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Key2" hidden="1">#REF!</definedName>
-    <definedName name="_khq3" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="_Ko2">#REF!</definedName>
     <definedName name="_Ko3">#REF!</definedName>
     <definedName name="_Ko4">#REF!</definedName>
     <definedName name="_Ko5">#REF!</definedName>
     <definedName name="_Ko6">#REF!</definedName>
     <definedName name="_Ko7">#REF!</definedName>
+    <definedName name="_khq3" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="_LAN3" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="_LC1">#REF!</definedName>
     <definedName name="_LC100">#REF!</definedName>
@@ -347,10 +347,6 @@
     <definedName name="CBWorkbookPriority" hidden="1">-604668737</definedName>
     <definedName name="Çdµ" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="CDPS">#REF!</definedName>
-    <definedName name="ChevronDim">#REF!</definedName>
-    <definedName name="chi" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="chitietbgiang2" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="chl" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="civil2" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="CLVC3">0.1</definedName>
     <definedName name="cn" hidden="1">{"'Sheet1'!$L$16"}</definedName>
@@ -387,6 +383,10 @@
     <definedName name="cur_3">#REF!</definedName>
     <definedName name="cur_4">#REF!</definedName>
     <definedName name="cus">#REF!</definedName>
+    <definedName name="ChevronDim">#REF!</definedName>
+    <definedName name="chi" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="chitietbgiang2" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="chl" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="D" localSheetId="0" hidden="1">{#N/A,#N/A,FALSE,"양식(을)"}</definedName>
     <definedName name="Ð" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="D_Name">"ドロップ 4"</definedName>
@@ -633,12 +633,12 @@
     <definedName name="GGG" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="gggg" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="ghf" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="gid" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="gj" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="gkd" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="gresg" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="GTOTAL" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="gthse" localSheetId="0" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
-    <definedName name="GTOTAL" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="gid" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="h" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="h_xoa" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="h_xoa2" hidden="1">{"'Sheet1'!$L$16"}</definedName>
@@ -732,12 +732,12 @@
     <definedName name="jsdjs" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="KCThep" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="KDJU" localSheetId="0" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
-    <definedName name="KH">#REF!</definedName>
-    <definedName name="khongtruotgia" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="ksbn" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="kshn" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="ksls" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="kt" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="KH">#REF!</definedName>
+    <definedName name="khongtruotgia" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="L_">#REF!</definedName>
     <definedName name="LadderSelect">#REF!</definedName>
     <definedName name="langson" hidden="1">{"'Sheet1'!$L$16"}</definedName>
@@ -762,8 +762,8 @@
     <definedName name="MA_CT">#REF!</definedName>
     <definedName name="MA_KH">#REF!</definedName>
     <definedName name="MA_SP">#REF!</definedName>
+    <definedName name="MA_TK">#REF!</definedName>
     <definedName name="Ma_the">#REF!</definedName>
-    <definedName name="MA_TK">#REF!</definedName>
     <definedName name="Ma_VT">#REF!</definedName>
     <definedName name="Mai" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="MAKH_CO">#REF!</definedName>
@@ -802,9 +802,6 @@
     <definedName name="NCC">#REF!</definedName>
     <definedName name="ND">#REF!</definedName>
     <definedName name="NEWNAME" localSheetId="0" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
-    <definedName name="ngu" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="nguyennha" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="NHAVESINH" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="nj" hidden="1">39</definedName>
     <definedName name="NMXFBZG" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="NO">#REF!</definedName>
@@ -818,14 +815,17 @@
     <definedName name="nuoc2" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="nuoùc" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="NXT">#REF!</definedName>
+    <definedName name="ngu" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="nguyennha" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="NHAVESINH" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="O">#REF!</definedName>
     <definedName name="õadfgdfgdf" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="ôclsaclnmc" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="OD">#REF!</definedName>
     <definedName name="ODH" hidden="1">#REF!</definedName>
     <definedName name="office" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="Outlet_Steam_Diameter18">#REF!</definedName>
     <definedName name="Outlet_Steam_Diameter20">#REF!</definedName>
+    <definedName name="ôclsaclnmc" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="P">#REF!</definedName>
     <definedName name="P.T.Xuan" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="P_NX">#REF!</definedName>
@@ -833,10 +833,6 @@
     <definedName name="PA2CAU39M" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="PauschalName">#REF!</definedName>
     <definedName name="pẻgtmaegnahr" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="ph" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="phantich3" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="Phieu">#REF!</definedName>
-    <definedName name="phuluc4" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="PIPING" hidden="1">#REF!</definedName>
     <definedName name="PKAAA" hidden="1">#REF!</definedName>
     <definedName name="PKBB" hidden="1">#REF!</definedName>
@@ -867,6 +863,10 @@
     <definedName name="ptich3" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="PUMP" localSheetId="0" hidden="1">{"A",#N/A,FALSE,"CALDERIN ";"A",#N/A,FALSE,"DIAM. EQ.CALD.";"A",#N/A,FALSE,"LONG.EF.CALD.";"A",#N/A,FALSE,"CIRCUNF. EF. CALD.";"A",#N/A,FALSE,"DIAG. EF. CALD.";"A",#N/A,FALSE,"MAX.DIAM.SIN REF.CALD.";"A",#N/A,FALSE,"CONEX. SHELL PL.";"A",#N/A,FALSE,"COMPENS.CALD."}</definedName>
     <definedName name="pvtot">#REF!</definedName>
+    <definedName name="ph" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="phantich3" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="Phieu">#REF!</definedName>
+    <definedName name="phuluc4" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="Q" localSheetId="0">{#N/A,#N/A,TRUE,"Basic";#N/A,#N/A,TRUE,"EXT-TABLE";#N/A,#N/A,TRUE,"STEEL";#N/A,#N/A,TRUE,"INT-Table";#N/A,#N/A,TRUE,"STEEL";#N/A,#N/A,TRUE,"Door"}</definedName>
     <definedName name="QANG" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="qd10_gt" hidden="1">{"'Sheet1'!$L$16"}</definedName>
@@ -894,8 +894,8 @@
     <definedName name="RRR" localSheetId="0" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="rrrrr" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="rrrrrrrr" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
+    <definedName name="RTYE" localSheetId="0" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="RTRE" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="RTYE" localSheetId="0" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="run">#REF!</definedName>
     <definedName name="RVI" hidden="1">#REF!</definedName>
     <definedName name="S" localSheetId="0" hidden="1">{#N/A,#N/A,FALSE,"Vessel1 1";#N/A,#N/A,FALSE,"Vessel1 2";#N/A,#N/A,FALSE,"Vessel1 3";#N/A,#N/A,FALSE,"Vessel1 4";#N/A,#N/A,FALSE,"Vessel1 5";#N/A,#N/A,FALSE,"Vessel1 6";#N/A,#N/A,FALSE,"Vessel1 7";#N/A,#N/A,FALSE,"Vessel1 8";#N/A,#N/A,FALSE,"Vessel1 9";#N/A,#N/A,FALSE,"Vessel1 10";#N/A,#N/A,FALSE,"Vessel1 11"}</definedName>
@@ -906,8 +906,8 @@
     <definedName name="Scrap_factor">#REF!</definedName>
     <definedName name="sd" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="SDFSF" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="sdsd" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="sđfsf" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="sdsd" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="Select">#REF!</definedName>
     <definedName name="sencount" hidden="1">2</definedName>
     <definedName name="SEP" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
@@ -979,17 +979,6 @@
     <definedName name="TextRefCopyRangeCount" hidden="1">21</definedName>
     <definedName name="TG_1">#REF!</definedName>
     <definedName name="TG_2">#REF!</definedName>
-    <definedName name="TH">#REF!</definedName>
-    <definedName name="TH_CN">#REF!</definedName>
-    <definedName name="TH_NO">#REF!</definedName>
-    <definedName name="TH_Z">#REF!</definedName>
-    <definedName name="tha" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="thang10" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="thanh" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="thdien" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="The">#REF!</definedName>
-    <definedName name="Thuong" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="thvt" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="tidf" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="TITLEBLOCK_CUSTOMERDOCNAME">#REF!</definedName>
     <definedName name="TITLEBLOCK_DOCUMENT">#REF!</definedName>
@@ -1161,10 +1150,6 @@
     <definedName name="total">[1]contactform!$U$59</definedName>
     <definedName name="TotalCases">#REF!</definedName>
     <definedName name="totalVAT">[1]contactform!$U$60</definedName>
-    <definedName name="tr" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="tralsmital1" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="TrangKH1A0" hidden="1">{"'Sheet1'!$L$16"}</definedName>
-    <definedName name="trw" localSheetId="0" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="tsfdsdf" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="TT_2">#REF!</definedName>
     <definedName name="ttt" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
@@ -1172,6 +1157,21 @@
     <definedName name="tygiagiam">#REF!</definedName>
     <definedName name="tygiatang">#REF!</definedName>
     <definedName name="TYJTJMMHJM" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="TH">#REF!</definedName>
+    <definedName name="TH_CN">#REF!</definedName>
+    <definedName name="TH_NO">#REF!</definedName>
+    <definedName name="TH_Z">#REF!</definedName>
+    <definedName name="tha" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="thang10" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="thanh" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="thdien" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="The">#REF!</definedName>
+    <definedName name="Thuong" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="thvt" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="tr" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="tralsmital1" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="TrangKH1A0" hidden="1">{"'Sheet1'!$L$16"}</definedName>
+    <definedName name="trw" localSheetId="0" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="UBDT" hidden="1">{"'Sheet1'!$L$16"}</definedName>
     <definedName name="UNI_FILT_OFFSPEC" hidden="1">2</definedName>
     <definedName name="UNI_FILT_ONSPEC" hidden="1">1</definedName>
@@ -1609,9 +1609,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="0_ "/>
   </numFmts>
   <fonts count="10">
@@ -1871,12 +1871,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1893,7 +1893,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1905,10 +1905,10 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="1" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1">
@@ -1917,7 +1917,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1932,36 +1932,207 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1969,183 +2140,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3104,21 +3098,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="40.5" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="39" t="s">
+      <c r="B1" s="52"/>
+      <c r="C1" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="40"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="44"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="65"/>
       <c r="L1" s="1" t="s">
         <v>1</v>
       </c>
@@ -3139,166 +3133,166 @@
       </c>
     </row>
     <row r="2" spans="1:17" ht="40.5" customHeight="1">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="48" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="49"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="27" t="s">
+      <c r="D2" s="70"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="M2" s="25" t="s">
+      <c r="M2" s="83" t="s">
         <v>44</v>
       </c>
-      <c r="N2" s="26" t="s">
+      <c r="N2" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="27"/>
-      <c r="P2" s="28"/>
-      <c r="Q2" s="27"/>
+      <c r="O2" s="56"/>
+      <c r="P2" s="85"/>
+      <c r="Q2" s="56"/>
     </row>
     <row r="3" spans="1:17" ht="22.7" customHeight="1">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="52" t="s">
+      <c r="B3" s="72"/>
+      <c r="C3" s="73" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="53"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="55" t="s">
+      <c r="D3" s="74"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="25"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="27"/>
-      <c r="P3" s="29"/>
-      <c r="Q3" s="27"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="56"/>
+      <c r="M3" s="83"/>
+      <c r="N3" s="84"/>
+      <c r="O3" s="56"/>
+      <c r="P3" s="86"/>
+      <c r="Q3" s="56"/>
     </row>
     <row r="4" spans="1:17" ht="22.7" customHeight="1">
-      <c r="A4" s="51"/>
-      <c r="B4" s="51"/>
-      <c r="C4" s="59" t="s">
+      <c r="A4" s="72"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="60"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="25"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="27"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="77"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="56"/>
+      <c r="M4" s="83"/>
+      <c r="N4" s="84"/>
+      <c r="O4" s="56"/>
+      <c r="P4" s="87"/>
+      <c r="Q4" s="56"/>
     </row>
     <row r="5" spans="1:17" ht="66" customHeight="1">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="33" t="s">
+      <c r="B5" s="52"/>
+      <c r="C5" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="32" t="s">
+      <c r="D5" s="54"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="27"/>
-      <c r="H5" s="36" t="s">
+      <c r="G5" s="56"/>
+      <c r="H5" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="I5" s="37"/>
-      <c r="J5" s="38"/>
+      <c r="I5" s="58"/>
+      <c r="J5" s="59"/>
       <c r="K5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="31" t="s">
+      <c r="L5" s="88" t="s">
         <v>36</v>
       </c>
-      <c r="M5" s="24"/>
+      <c r="M5" s="82"/>
       <c r="N5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="23" t="s">
+      <c r="O5" s="81" t="s">
         <v>46</v>
       </c>
-      <c r="P5" s="24"/>
-      <c r="Q5" s="24"/>
+      <c r="P5" s="82"/>
+      <c r="Q5" s="82"/>
     </row>
     <row r="6" spans="1:17" ht="18.600000000000001" customHeight="1">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="62" t="s">
+      <c r="C6" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="64" t="s">
+      <c r="D6" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="65"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="62" t="s">
+      <c r="E6" s="51"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="62" t="s">
+      <c r="H6" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="62" t="s">
+      <c r="I6" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="J6" s="62" t="s">
+      <c r="J6" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="62" t="s">
+      <c r="K6" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="62" t="s">
+      <c r="L6" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="M6" s="62" t="s">
+      <c r="M6" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="N6" s="62" t="s">
+      <c r="N6" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="O6" s="62" t="s">
+      <c r="O6" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="P6" s="68" t="s">
+      <c r="P6" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="Q6" s="56"/>
+      <c r="Q6" s="24"/>
     </row>
     <row r="7" spans="1:17" ht="21.6" customHeight="1">
-      <c r="A7" s="63"/>
-      <c r="B7" s="63"/>
-      <c r="C7" s="63"/>
+      <c r="A7" s="50"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="50"/>
       <c r="D7" s="1" t="s">
         <v>29</v>
       </c>
@@ -3308,46 +3302,46 @@
       <c r="F7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
-      <c r="J7" s="63"/>
-      <c r="K7" s="63"/>
-      <c r="L7" s="63"/>
-      <c r="M7" s="63"/>
-      <c r="N7" s="63"/>
-      <c r="O7" s="63"/>
-      <c r="P7" s="69"/>
-      <c r="Q7" s="58"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="50"/>
+      <c r="J7" s="50"/>
+      <c r="K7" s="50"/>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
+      <c r="N7" s="50"/>
+      <c r="O7" s="50"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="26"/>
     </row>
     <row r="8" spans="1:17" ht="16.899999999999999" customHeight="1">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="90"/>
-      <c r="N8" s="90"/>
-      <c r="O8" s="21"/>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="21"/>
+      <c r="N8" s="21"/>
+      <c r="O8" s="20"/>
+      <c r="P8" s="29"/>
+      <c r="Q8" s="30"/>
     </row>
     <row r="9" spans="1:17" ht="24.95" customHeight="1">
       <c r="A9" s="4"/>
       <c r="B9" s="5"/>
-      <c r="C9" s="70" t="s">
+      <c r="C9" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="70"/>
-      <c r="E9" s="70"/>
-      <c r="F9" s="71"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="28"/>
       <c r="G9" s="6"/>
       <c r="H9" s="7"/>
       <c r="I9" s="6">
@@ -3362,18 +3356,18 @@
         <v>0</v>
       </c>
       <c r="O9" s="11"/>
-      <c r="P9" s="64"/>
-      <c r="Q9" s="66"/>
+      <c r="P9" s="29"/>
+      <c r="Q9" s="30"/>
     </row>
     <row r="10" spans="1:17" ht="24.95" customHeight="1">
       <c r="A10" s="12"/>
       <c r="B10" s="13"/>
-      <c r="C10" s="72" t="s">
+      <c r="C10" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="72"/>
-      <c r="E10" s="72"/>
-      <c r="F10" s="73"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="32"/>
       <c r="G10" s="6"/>
       <c r="H10" s="3"/>
       <c r="I10" s="6"/>
@@ -3383,152 +3377,183 @@
       <c r="M10" s="3"/>
       <c r="N10" s="14"/>
       <c r="O10" s="15"/>
-      <c r="P10" s="64"/>
-      <c r="Q10" s="66"/>
+      <c r="P10" s="29"/>
+      <c r="Q10" s="30"/>
     </row>
     <row r="11" spans="1:17" ht="27" customHeight="1">
-      <c r="A11" s="74" t="s">
+      <c r="A11" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="75"/>
-      <c r="C11" s="75"/>
-      <c r="D11" s="75"/>
-      <c r="E11" s="75"/>
-      <c r="F11" s="75"/>
-      <c r="G11" s="75"/>
-      <c r="H11" s="75"/>
-      <c r="I11" s="75"/>
-      <c r="J11" s="75"/>
-      <c r="K11" s="80" t="s">
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
+      <c r="K11" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="80"/>
-      <c r="M11" s="80"/>
-      <c r="N11" s="80"/>
-      <c r="O11" s="80"/>
-      <c r="P11" s="80"/>
-      <c r="Q11" s="81"/>
+      <c r="L11" s="39"/>
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="39"/>
+      <c r="P11" s="39"/>
+      <c r="Q11" s="40"/>
     </row>
     <row r="12" spans="1:17" ht="27" customHeight="1">
-      <c r="A12" s="76"/>
-      <c r="B12" s="77"/>
-      <c r="C12" s="77"/>
-      <c r="D12" s="77"/>
-      <c r="E12" s="77"/>
-      <c r="F12" s="77"/>
-      <c r="G12" s="77"/>
-      <c r="H12" s="77"/>
-      <c r="I12" s="77"/>
-      <c r="J12" s="77"/>
-      <c r="K12" s="82"/>
-      <c r="L12" s="82"/>
-      <c r="M12" s="82"/>
-      <c r="N12" s="82"/>
-      <c r="O12" s="82"/>
-      <c r="P12" s="82"/>
-      <c r="Q12" s="83"/>
+      <c r="A12" s="35"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="41"/>
+      <c r="L12" s="41"/>
+      <c r="M12" s="41"/>
+      <c r="N12" s="41"/>
+      <c r="O12" s="41"/>
+      <c r="P12" s="41"/>
+      <c r="Q12" s="42"/>
     </row>
     <row r="13" spans="1:17" ht="27" customHeight="1">
-      <c r="A13" s="76"/>
-      <c r="B13" s="77"/>
-      <c r="C13" s="77"/>
-      <c r="D13" s="77"/>
-      <c r="E13" s="77"/>
-      <c r="F13" s="77"/>
-      <c r="G13" s="77"/>
-      <c r="H13" s="77"/>
-      <c r="I13" s="77"/>
-      <c r="J13" s="77"/>
-      <c r="K13" s="84"/>
-      <c r="L13" s="84"/>
-      <c r="M13" s="84"/>
-      <c r="N13" s="85" t="s">
+      <c r="A13" s="35"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="36"/>
+      <c r="K13" s="43"/>
+      <c r="L13" s="43"/>
+      <c r="M13" s="43"/>
+      <c r="N13" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="O13" s="86"/>
-      <c r="P13" s="86"/>
-      <c r="Q13" s="87"/>
+      <c r="O13" s="45"/>
+      <c r="P13" s="45"/>
+      <c r="Q13" s="46"/>
     </row>
     <row r="14" spans="1:17" ht="27" customHeight="1">
-      <c r="A14" s="76"/>
-      <c r="B14" s="77"/>
-      <c r="C14" s="77"/>
-      <c r="D14" s="77"/>
-      <c r="E14" s="77"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="77"/>
-      <c r="H14" s="77"/>
-      <c r="I14" s="77"/>
-      <c r="J14" s="77"/>
-      <c r="K14" s="86" t="s">
+      <c r="A14" s="35"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="36"/>
+      <c r="J14" s="36"/>
+      <c r="K14" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="L14" s="86"/>
-      <c r="M14" s="86"/>
-      <c r="N14" s="86"/>
-      <c r="O14" s="86"/>
-      <c r="P14" s="86"/>
-      <c r="Q14" s="87"/>
+      <c r="L14" s="45"/>
+      <c r="M14" s="45"/>
+      <c r="N14" s="45"/>
+      <c r="O14" s="45"/>
+      <c r="P14" s="45"/>
+      <c r="Q14" s="46"/>
     </row>
     <row r="15" spans="1:17" ht="255" customHeight="1">
-      <c r="A15" s="78"/>
-      <c r="B15" s="79"/>
-      <c r="C15" s="79"/>
-      <c r="D15" s="79"/>
-      <c r="E15" s="79"/>
-      <c r="F15" s="79"/>
-      <c r="G15" s="79"/>
-      <c r="H15" s="79"/>
-      <c r="I15" s="79"/>
-      <c r="J15" s="79"/>
-      <c r="K15" s="88"/>
-      <c r="L15" s="88"/>
-      <c r="M15" s="88"/>
-      <c r="N15" s="88"/>
-      <c r="O15" s="88"/>
-      <c r="P15" s="88"/>
-      <c r="Q15" s="89"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="47"/>
+      <c r="L15" s="47"/>
+      <c r="M15" s="47"/>
+      <c r="N15" s="47"/>
+      <c r="O15" s="47"/>
+      <c r="P15" s="47"/>
+      <c r="Q15" s="48"/>
     </row>
     <row r="16" spans="1:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="A16" s="67"/>
-      <c r="B16" s="67"/>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
       <c r="E16" s="16"/>
-      <c r="F16" s="67"/>
-      <c r="G16" s="67"/>
-      <c r="H16" s="67"/>
-      <c r="I16" s="67"/>
-      <c r="J16" s="67"/>
-      <c r="K16" s="67"/>
-      <c r="L16" s="67"/>
-      <c r="M16" s="67"/>
-      <c r="N16" s="67"/>
-      <c r="O16" s="67"/>
-      <c r="P16" s="67"/>
-      <c r="Q16" s="67"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="22"/>
+      <c r="Q16" s="22"/>
     </row>
     <row r="17" spans="1:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="A17" s="67"/>
-      <c r="B17" s="67"/>
-      <c r="C17" s="67"/>
-      <c r="D17" s="67"/>
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
       <c r="E17" s="16"/>
-      <c r="F17" s="67"/>
-      <c r="G17" s="67"/>
-      <c r="H17" s="67"/>
-      <c r="I17" s="67"/>
-      <c r="J17" s="67"/>
-      <c r="K17" s="67"/>
-      <c r="L17" s="67"/>
-      <c r="M17" s="67"/>
-      <c r="N17" s="67"/>
-      <c r="O17" s="67"/>
-      <c r="P17" s="67"/>
-      <c r="Q17" s="67"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="22"/>
+      <c r="Q17" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="47">
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="M2:M4"/>
+    <mergeCell ref="N2:N4"/>
+    <mergeCell ref="O2:O4"/>
+    <mergeCell ref="P2:P4"/>
+    <mergeCell ref="Q2:Q4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L2:L4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="F1:K2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="A3:B4"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F3:K4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="G6:G7"/>
     <mergeCell ref="A16:D17"/>
     <mergeCell ref="F16:Q17"/>
     <mergeCell ref="P6:Q7"/>
@@ -3545,36 +3570,6 @@
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="L6:L7"/>
     <mergeCell ref="M6:M7"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="O6:O7"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:K2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A3:B4"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="F3:K4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="M2:M4"/>
-    <mergeCell ref="N2:N4"/>
-    <mergeCell ref="O2:O4"/>
-    <mergeCell ref="P2:P4"/>
-    <mergeCell ref="Q2:Q4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L2:L4"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="49" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Handle function add more infomation of item (Heat, ID_Code) V3 and Update Icon for app
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/po_template.xlsx
+++ b/MPR_Managerment/Templates/po_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Git\MPR_Managerment\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c02630c4a1efac79/Working/Final_Project_DLHI_Management/MPR_Managerment/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7353541E-4729-457E-AF31-1D8DE9DEACD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{7353541E-4729-457E-AF31-1D8DE9DEACD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{292C2B6B-114D-47C8-89F2-C16AE4B10DC6}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="225" windowWidth="29040" windowHeight="15720" xr2:uid="{08BC6B50-49E0-41CF-A464-82D4FBAF0A1C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{08BC6B50-49E0-41CF-A464-82D4FBAF0A1C}"/>
   </bookViews>
   <sheets>
     <sheet name="DV-DPCII-PC-9" sheetId="1" r:id="rId1"/>
@@ -1362,21 +1362,10 @@
     <definedName name="ㅛㅛㅛ" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="実行" hidden="1">{"'Sheet1'!$L$16"}</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1422,9 +1411,6 @@
     <t>Work Order No.
 (수주통보서 번호)</t>
     <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>PHẠM MẠNH HOÀNG</t>
   </si>
   <si>
     <t>M.P.R No. (요구서 번호)
@@ -1609,23 +1595,26 @@
   <si>
     <t>DLHI Viet Nam</t>
   </si>
+  <si>
+    <t>&lt;&lt;USER_NAME&gt;&gt;</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0_ "/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1685,7 +1674,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1885,11 +1874,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1908,7 +1897,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1920,10 +1909,10 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="1" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1">
@@ -1953,39 +1942,156 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2039,123 +2145,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -3095,40 +3084,40 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q17"/>
-  <sheetFormatPr defaultColWidth="9.875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.125" style="2" customWidth="1"/>
-    <col min="4" max="6" width="13.125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="9.875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="11.875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="12.375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="28.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.625" style="2" customWidth="1"/>
-    <col min="12" max="13" width="15.375" style="2" customWidth="1"/>
-    <col min="14" max="15" width="18.625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="15.375" style="2" customWidth="1"/>
-    <col min="17" max="17" width="15.375" style="17" customWidth="1"/>
-    <col min="18" max="16384" width="9.875" style="2"/>
+    <col min="1" max="1" width="5.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="2" customWidth="1"/>
+    <col min="4" max="6" width="13.140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="12.42578125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="28.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" style="2" customWidth="1"/>
+    <col min="12" max="13" width="15.42578125" style="2" customWidth="1"/>
+    <col min="14" max="15" width="18.5703125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="15.42578125" style="2" customWidth="1"/>
+    <col min="17" max="17" width="15.42578125" style="17" customWidth="1"/>
+    <col min="18" max="16384" width="9.85546875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="40.5" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="59" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="60"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="64"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="43"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="47"/>
       <c r="L1" s="1" t="s">
         <v>1</v>
       </c>
@@ -3149,186 +3138,186 @@
       </c>
     </row>
     <row r="2" spans="1:17" ht="40.5" customHeight="1">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="68" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="69"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="55" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="51" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="52"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="M2" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="M2" s="82" t="s">
-        <v>44</v>
-      </c>
-      <c r="N2" s="83" t="s">
-        <v>8</v>
-      </c>
-      <c r="O2" s="55"/>
-      <c r="P2" s="84"/>
-      <c r="Q2" s="55"/>
+      <c r="N2" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="O2" s="28"/>
+      <c r="P2" s="29"/>
+      <c r="Q2" s="28"/>
     </row>
     <row r="3" spans="1:17" ht="22.7" customHeight="1">
-      <c r="A3" s="71" t="s">
+      <c r="A3" s="54" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="54"/>
+      <c r="C3" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="56"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="71"/>
-      <c r="C3" s="72" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="73"/>
-      <c r="E3" s="74"/>
-      <c r="F3" s="75" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="75"/>
-      <c r="J3" s="75"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="55"/>
-      <c r="M3" s="82"/>
-      <c r="N3" s="83"/>
-      <c r="O3" s="55"/>
-      <c r="P3" s="85"/>
-      <c r="Q3" s="55"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="27"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="30"/>
+      <c r="Q3" s="28"/>
     </row>
     <row r="4" spans="1:17" ht="22.7" customHeight="1">
-      <c r="A4" s="71"/>
-      <c r="B4" s="71"/>
-      <c r="C4" s="77" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="78"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="76"/>
-      <c r="I4" s="76"/>
-      <c r="J4" s="76"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="82"/>
-      <c r="N4" s="83"/>
-      <c r="O4" s="55"/>
-      <c r="P4" s="86"/>
-      <c r="Q4" s="55"/>
+      <c r="A4" s="54"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="62" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="63"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60"/>
+      <c r="H4" s="60"/>
+      <c r="I4" s="60"/>
+      <c r="J4" s="60"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="28"/>
     </row>
     <row r="5" spans="1:17" ht="66" customHeight="1">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="35"/>
+      <c r="C5" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="52" t="s">
+      <c r="D5" s="37"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="53"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="51" t="s">
+      <c r="G5" s="28"/>
+      <c r="H5" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="I5" s="40"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="55"/>
-      <c r="H5" s="56" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="57"/>
-      <c r="J5" s="58"/>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5" s="25"/>
+      <c r="N5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="87" t="s">
-        <v>36</v>
-      </c>
-      <c r="M5" s="81"/>
-      <c r="N5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="O5" s="80" t="s">
-        <v>46</v>
-      </c>
-      <c r="P5" s="81"/>
-      <c r="Q5" s="81"/>
+      <c r="O5" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="P5" s="25"/>
+      <c r="Q5" s="25"/>
     </row>
     <row r="6" spans="1:17" ht="18.600000000000001" customHeight="1">
-      <c r="A6" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="21" t="s">
+      <c r="A6" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="D6" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="E6" s="65"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="50"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="21" t="s">
+      <c r="H6" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="I6" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="J6" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="J6" s="21" t="s">
+      <c r="K6" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="21" t="s">
+      <c r="L6" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="21" t="s">
+      <c r="M6" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="M6" s="21" t="s">
+      <c r="N6" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="N6" s="21" t="s">
+      <c r="O6" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="O6" s="21" t="s">
+      <c r="P6" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="P6" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q6" s="25"/>
+      <c r="Q6" s="59"/>
     </row>
     <row r="7" spans="1:17" ht="21.6" customHeight="1">
-      <c r="A7" s="22"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
+      <c r="A7" s="34"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
       <c r="D7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="26"/>
-      <c r="Q7" s="27"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="34"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="34"/>
+      <c r="P7" s="68"/>
+      <c r="Q7" s="61"/>
     </row>
     <row r="8" spans="1:17" ht="16.899999999999999" customHeight="1">
       <c r="A8" s="19"/>
@@ -3342,26 +3331,26 @@
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
       <c r="K8" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="L8" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="L8" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="M8" s="20"/>
       <c r="N8" s="20"/>
       <c r="O8" s="19"/>
-      <c r="P8" s="30"/>
-      <c r="Q8" s="31"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="23"/>
     </row>
     <row r="9" spans="1:17" ht="24.95" customHeight="1">
       <c r="A9" s="4"/>
       <c r="B9" s="5"/>
-      <c r="C9" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="29"/>
+      <c r="C9" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="69"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="70"/>
       <c r="G9" s="6"/>
       <c r="H9" s="7"/>
       <c r="I9" s="6">
@@ -3376,18 +3365,18 @@
         <v>0</v>
       </c>
       <c r="O9" s="11"/>
-      <c r="P9" s="30"/>
-      <c r="Q9" s="31"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="23"/>
     </row>
     <row r="10" spans="1:17" ht="24.95" customHeight="1">
       <c r="A10" s="12"/>
       <c r="B10" s="13"/>
-      <c r="C10" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="33"/>
+      <c r="C10" s="71" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="71"/>
+      <c r="E10" s="71"/>
+      <c r="F10" s="72"/>
       <c r="G10" s="6"/>
       <c r="H10" s="3"/>
       <c r="I10" s="6"/>
@@ -3395,185 +3384,154 @@
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
-      <c r="N10" s="88"/>
+      <c r="N10" s="21"/>
       <c r="O10" s="14"/>
-      <c r="P10" s="30"/>
-      <c r="Q10" s="31"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="23"/>
     </row>
     <row r="11" spans="1:17" ht="27" customHeight="1">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="73" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="74"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
+      <c r="I11" s="74"/>
+      <c r="J11" s="74"/>
+      <c r="K11" s="79" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="40" t="s">
-        <v>34</v>
-      </c>
-      <c r="L11" s="40"/>
-      <c r="M11" s="40"/>
-      <c r="N11" s="40"/>
-      <c r="O11" s="40"/>
-      <c r="P11" s="40"/>
-      <c r="Q11" s="41"/>
+      <c r="L11" s="79"/>
+      <c r="M11" s="79"/>
+      <c r="N11" s="79"/>
+      <c r="O11" s="79"/>
+      <c r="P11" s="79"/>
+      <c r="Q11" s="80"/>
     </row>
     <row r="12" spans="1:17" ht="27" customHeight="1">
-      <c r="A12" s="36"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="37"/>
-      <c r="H12" s="37"/>
-      <c r="I12" s="37"/>
-      <c r="J12" s="37"/>
-      <c r="K12" s="42"/>
-      <c r="L12" s="42"/>
-      <c r="M12" s="42"/>
-      <c r="N12" s="42"/>
-      <c r="O12" s="42"/>
-      <c r="P12" s="42"/>
-      <c r="Q12" s="43"/>
+      <c r="A12" s="75"/>
+      <c r="B12" s="76"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="76"/>
+      <c r="F12" s="76"/>
+      <c r="G12" s="76"/>
+      <c r="H12" s="76"/>
+      <c r="I12" s="76"/>
+      <c r="J12" s="76"/>
+      <c r="K12" s="81"/>
+      <c r="L12" s="81"/>
+      <c r="M12" s="81"/>
+      <c r="N12" s="81"/>
+      <c r="O12" s="81"/>
+      <c r="P12" s="81"/>
+      <c r="Q12" s="82"/>
     </row>
     <row r="13" spans="1:17" ht="27" customHeight="1">
-      <c r="A13" s="36"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="37"/>
-      <c r="K13" s="44"/>
-      <c r="L13" s="44"/>
-      <c r="M13" s="44"/>
-      <c r="N13" s="45" t="s">
-        <v>44</v>
-      </c>
-      <c r="O13" s="46"/>
-      <c r="P13" s="46"/>
-      <c r="Q13" s="47"/>
+      <c r="A13" s="75"/>
+      <c r="B13" s="76"/>
+      <c r="C13" s="76"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="76"/>
+      <c r="F13" s="76"/>
+      <c r="G13" s="76"/>
+      <c r="H13" s="76"/>
+      <c r="I13" s="76"/>
+      <c r="J13" s="76"/>
+      <c r="K13" s="83"/>
+      <c r="L13" s="83"/>
+      <c r="M13" s="83"/>
+      <c r="N13" s="84" t="s">
+        <v>43</v>
+      </c>
+      <c r="O13" s="85"/>
+      <c r="P13" s="85"/>
+      <c r="Q13" s="86"/>
     </row>
     <row r="14" spans="1:17" ht="27" customHeight="1">
-      <c r="A14" s="36"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
-      <c r="J14" s="37"/>
-      <c r="K14" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="L14" s="46"/>
-      <c r="M14" s="46"/>
-      <c r="N14" s="46"/>
-      <c r="O14" s="46"/>
-      <c r="P14" s="46"/>
-      <c r="Q14" s="47"/>
+      <c r="A14" s="75"/>
+      <c r="B14" s="76"/>
+      <c r="C14" s="76"/>
+      <c r="D14" s="76"/>
+      <c r="E14" s="76"/>
+      <c r="F14" s="76"/>
+      <c r="G14" s="76"/>
+      <c r="H14" s="76"/>
+      <c r="I14" s="76"/>
+      <c r="J14" s="76"/>
+      <c r="K14" s="85" t="s">
+        <v>34</v>
+      </c>
+      <c r="L14" s="85"/>
+      <c r="M14" s="85"/>
+      <c r="N14" s="85"/>
+      <c r="O14" s="85"/>
+      <c r="P14" s="85"/>
+      <c r="Q14" s="86"/>
     </row>
     <row r="15" spans="1:17" ht="255" customHeight="1">
-      <c r="A15" s="38"/>
-      <c r="B15" s="39"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="39"/>
-      <c r="J15" s="39"/>
-      <c r="K15" s="48"/>
-      <c r="L15" s="48"/>
-      <c r="M15" s="48"/>
-      <c r="N15" s="48"/>
-      <c r="O15" s="48"/>
-      <c r="P15" s="48"/>
-      <c r="Q15" s="49"/>
+      <c r="A15" s="77"/>
+      <c r="B15" s="78"/>
+      <c r="C15" s="78"/>
+      <c r="D15" s="78"/>
+      <c r="E15" s="78"/>
+      <c r="F15" s="78"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="78"/>
+      <c r="J15" s="78"/>
+      <c r="K15" s="87"/>
+      <c r="L15" s="87"/>
+      <c r="M15" s="87"/>
+      <c r="N15" s="87"/>
+      <c r="O15" s="87"/>
+      <c r="P15" s="87"/>
+      <c r="Q15" s="88"/>
     </row>
     <row r="16" spans="1:17" s="16" customFormat="1" ht="15" customHeight="1">
-      <c r="A16" s="23"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
+      <c r="A16" s="66"/>
+      <c r="B16" s="66"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
       <c r="E16" s="15"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
+      <c r="F16" s="66"/>
+      <c r="G16" s="66"/>
+      <c r="H16" s="66"/>
+      <c r="I16" s="66"/>
+      <c r="J16" s="66"/>
+      <c r="K16" s="66"/>
+      <c r="L16" s="66"/>
+      <c r="M16" s="66"/>
+      <c r="N16" s="66"/>
+      <c r="O16" s="66"/>
+      <c r="P16" s="66"/>
+      <c r="Q16" s="66"/>
     </row>
     <row r="17" spans="1:17" s="16" customFormat="1" ht="15" customHeight="1">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
+      <c r="A17" s="66"/>
+      <c r="B17" s="66"/>
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
       <c r="E17" s="15"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="23"/>
-      <c r="O17" s="23"/>
-      <c r="P17" s="23"/>
-      <c r="Q17" s="23"/>
+      <c r="F17" s="66"/>
+      <c r="G17" s="66"/>
+      <c r="H17" s="66"/>
+      <c r="I17" s="66"/>
+      <c r="J17" s="66"/>
+      <c r="K17" s="66"/>
+      <c r="L17" s="66"/>
+      <c r="M17" s="66"/>
+      <c r="N17" s="66"/>
+      <c r="O17" s="66"/>
+      <c r="P17" s="66"/>
+      <c r="Q17" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="M2:M4"/>
-    <mergeCell ref="N2:N4"/>
-    <mergeCell ref="O2:O4"/>
-    <mergeCell ref="P2:P4"/>
-    <mergeCell ref="Q2:Q4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L2:L4"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="O6:O7"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:K2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A3:B4"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="F3:K4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="H6:H7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="A16:D17"/>
@@ -3590,9 +3548,40 @@
     <mergeCell ref="K14:Q15"/>
     <mergeCell ref="J6:J7"/>
     <mergeCell ref="K6:K7"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="F1:K2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="A3:B4"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F3:K4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="M2:M4"/>
+    <mergeCell ref="N2:N4"/>
+    <mergeCell ref="O2:O4"/>
+    <mergeCell ref="P2:P4"/>
+    <mergeCell ref="Q2:Q4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L2:L4"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="46" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="49" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
hiển thị thông báo Loading
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/po_template.xlsx
+++ b/MPR_Managerment/Templates/po_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Management\MPR_Managerment\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Git\MPR_Managerment\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282DC735-5FC6-44D0-9D3F-889F4E719322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{059E7AFC-105C-406E-BC84-A66D9F6B13E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="735" windowWidth="29040" windowHeight="15720" xr2:uid="{08BC6B50-49E0-41CF-A464-82D4FBAF0A1C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{08BC6B50-49E0-41CF-A464-82D4FBAF0A1C}"/>
   </bookViews>
   <sheets>
     <sheet name="DV-DPCII-PC-9" sheetId="1" r:id="rId1"/>
@@ -1362,10 +1362,21 @@
     <definedName name="ㅛㅛㅛ" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="実行" hidden="1">{"'Sheet1'!$L$16"}</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1604,17 +1615,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="0_ "/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0_ "/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1632,7 +1643,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1665,7 +1676,7 @@
     <font>
       <sz val="11"/>
       <color theme="2" tint="-0.89999084444715716"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1891,17 +1902,125 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="1" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1920,11 +2039,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1935,27 +2057,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1974,129 +2075,66 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2115,38 +2153,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="5" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -3086,485 +3112,454 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q17"/>
-  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" style="9" customWidth="1"/>
-    <col min="4" max="6" width="13.140625" style="9" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" style="9" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" style="9" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" style="9" customWidth="1"/>
-    <col min="10" max="10" width="28.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" style="9" customWidth="1"/>
-    <col min="12" max="13" width="15.42578125" style="9" customWidth="1"/>
-    <col min="14" max="15" width="18.5703125" style="9" customWidth="1"/>
-    <col min="16" max="16" width="15.42578125" style="9" customWidth="1"/>
-    <col min="17" max="17" width="15.42578125" style="80" customWidth="1"/>
-    <col min="18" max="16384" width="9.85546875" style="9"/>
+    <col min="1" max="1" width="5.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.125" style="2" customWidth="1"/>
+    <col min="4" max="6" width="13.125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="9.875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="11.875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="12.375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="28.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.625" style="88" customWidth="1"/>
+    <col min="12" max="13" width="15.375" style="2" customWidth="1"/>
+    <col min="14" max="15" width="18.625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="15.375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="15.375" style="21" customWidth="1"/>
+    <col min="18" max="16384" width="9.875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="40.5" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="8" t="s">
+      <c r="D1" s="39"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="40.5" customHeight="1">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="10" t="s">
+      <c r="B2" s="24"/>
+      <c r="C2" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="16" t="s">
+      <c r="D2" s="48"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="M2" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="N2" s="18" t="s">
+      <c r="N2" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="O2" s="16"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="16"/>
+      <c r="O2" s="25"/>
+      <c r="P2" s="28"/>
+      <c r="Q2" s="25"/>
     </row>
     <row r="3" spans="1:17" ht="22.7" customHeight="1">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="21" t="s">
+      <c r="B3" s="50"/>
+      <c r="C3" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="22"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="24" t="s">
+      <c r="D3" s="52"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="16"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="55"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="27"/>
+      <c r="O3" s="25"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="25"/>
     </row>
     <row r="4" spans="1:17" ht="22.7" customHeight="1">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="81" t="s">
+      <c r="A4" s="50"/>
+      <c r="B4" s="50"/>
+      <c r="C4" s="58" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="82"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="16"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="57"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="25"/>
+      <c r="P4" s="30"/>
+      <c r="Q4" s="25"/>
     </row>
     <row r="5" spans="1:17" ht="66" customHeight="1">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="30" t="s">
+      <c r="B5" s="24"/>
+      <c r="C5" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="31"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="1" t="s">
+      <c r="D5" s="35"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="33" t="s">
+      <c r="G5" s="25"/>
+      <c r="H5" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="I5" s="34"/>
-      <c r="J5" s="35"/>
-      <c r="K5" s="8" t="s">
+      <c r="I5" s="37"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="36" t="s">
+      <c r="L5" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="M5" s="16"/>
-      <c r="N5" s="8" t="s">
+      <c r="M5" s="25"/>
+      <c r="N5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="O5" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
+      <c r="P5" s="25"/>
+      <c r="Q5" s="25"/>
     </row>
     <row r="6" spans="1:17" ht="18.600000000000001" customHeight="1">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="33" t="s">
+      <c r="D6" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="34"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="37" t="s">
+      <c r="E6" s="37"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="37" t="s">
+      <c r="H6" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="37" t="s">
+      <c r="I6" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="37" t="s">
+      <c r="J6" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="37" t="s">
+      <c r="K6" s="85" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="37" t="s">
+      <c r="L6" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="M6" s="37" t="s">
+      <c r="M6" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="N6" s="37" t="s">
+      <c r="N6" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="O6" s="37" t="s">
+      <c r="O6" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="P6" s="38" t="s">
+      <c r="P6" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="Q6" s="25"/>
+      <c r="Q6" s="55"/>
     </row>
     <row r="7" spans="1:17" ht="21.6" customHeight="1">
-      <c r="A7" s="39"/>
-      <c r="B7" s="39"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="8" t="s">
+      <c r="A7" s="33"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="39"/>
-      <c r="K7" s="39"/>
-      <c r="L7" s="39"/>
-      <c r="M7" s="39"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="39"/>
-      <c r="P7" s="40"/>
-      <c r="Q7" s="28"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="33"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="86"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="33"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="63"/>
+      <c r="Q7" s="57"/>
     </row>
     <row r="8" spans="1:17" ht="16.899999999999999" customHeight="1">
-      <c r="A8" s="41"/>
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="41"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="41" t="s">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="87" t="s">
         <v>46</v>
       </c>
-      <c r="L8" s="41" t="s">
+      <c r="L8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="M8" s="43"/>
-      <c r="N8" s="43"/>
-      <c r="O8" s="41"/>
-      <c r="P8" s="33"/>
-      <c r="Q8" s="35"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="23"/>
     </row>
     <row r="9" spans="1:17" ht="24.95" customHeight="1">
-      <c r="A9" s="44"/>
-      <c r="B9" s="45"/>
-      <c r="C9" s="46" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="47"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="48">
+      <c r="D9" s="64"/>
+      <c r="E9" s="64"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="10">
         <v>0</v>
       </c>
-      <c r="J9" s="50"/>
-      <c r="K9" s="51"/>
-      <c r="L9" s="50"/>
-      <c r="M9" s="52"/>
-      <c r="N9" s="53">
+      <c r="J9" s="3"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="13">
         <f>SUM(N8:N8)</f>
         <v>0</v>
       </c>
-      <c r="O9" s="54"/>
-      <c r="P9" s="33"/>
-      <c r="Q9" s="35"/>
+      <c r="O9" s="14"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="23"/>
     </row>
     <row r="10" spans="1:17" ht="24.95" customHeight="1">
-      <c r="A10" s="55"/>
-      <c r="B10" s="56"/>
-      <c r="C10" s="57" t="s">
+      <c r="A10" s="15"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="66" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="58"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="50"/>
-      <c r="I10" s="48"/>
-      <c r="J10" s="50"/>
-      <c r="K10" s="50"/>
-      <c r="L10" s="50"/>
-      <c r="M10" s="50"/>
-      <c r="N10" s="59"/>
-      <c r="O10" s="60"/>
-      <c r="P10" s="33"/>
-      <c r="Q10" s="35"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="67"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="23"/>
     </row>
     <row r="11" spans="1:17" ht="27" customHeight="1">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="62"/>
-      <c r="C11" s="62"/>
-      <c r="D11" s="62"/>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62"/>
-      <c r="H11" s="62"/>
-      <c r="I11" s="62"/>
-      <c r="J11" s="62"/>
-      <c r="K11" s="63" t="s">
+      <c r="B11" s="69"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="L11" s="63"/>
-      <c r="M11" s="63"/>
-      <c r="N11" s="63"/>
-      <c r="O11" s="63"/>
-      <c r="P11" s="63"/>
-      <c r="Q11" s="64"/>
+      <c r="L11" s="74"/>
+      <c r="M11" s="74"/>
+      <c r="N11" s="74"/>
+      <c r="O11" s="74"/>
+      <c r="P11" s="74"/>
+      <c r="Q11" s="75"/>
     </row>
     <row r="12" spans="1:17" ht="27" customHeight="1">
-      <c r="A12" s="65"/>
-      <c r="B12" s="66"/>
-      <c r="C12" s="66"/>
-      <c r="D12" s="66"/>
-      <c r="E12" s="66"/>
-      <c r="F12" s="66"/>
-      <c r="G12" s="66"/>
-      <c r="H12" s="66"/>
-      <c r="I12" s="66"/>
-      <c r="J12" s="66"/>
-      <c r="K12" s="67"/>
-      <c r="L12" s="67"/>
-      <c r="M12" s="67"/>
-      <c r="N12" s="67"/>
-      <c r="O12" s="67"/>
-      <c r="P12" s="67"/>
-      <c r="Q12" s="68"/>
+      <c r="A12" s="70"/>
+      <c r="B12" s="71"/>
+      <c r="C12" s="71"/>
+      <c r="D12" s="71"/>
+      <c r="E12" s="71"/>
+      <c r="F12" s="71"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="71"/>
+      <c r="I12" s="71"/>
+      <c r="J12" s="71"/>
+      <c r="K12" s="76"/>
+      <c r="L12" s="76"/>
+      <c r="M12" s="76"/>
+      <c r="N12" s="76"/>
+      <c r="O12" s="76"/>
+      <c r="P12" s="76"/>
+      <c r="Q12" s="77"/>
     </row>
     <row r="13" spans="1:17" ht="27" customHeight="1">
-      <c r="A13" s="65"/>
-      <c r="B13" s="66"/>
-      <c r="C13" s="66"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="66"/>
-      <c r="F13" s="66"/>
-      <c r="G13" s="66"/>
-      <c r="H13" s="66"/>
-      <c r="I13" s="66"/>
-      <c r="J13" s="66"/>
-      <c r="K13" s="69"/>
-      <c r="L13" s="69"/>
-      <c r="M13" s="69"/>
-      <c r="N13" s="70" t="s">
+      <c r="A13" s="70"/>
+      <c r="B13" s="71"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="71"/>
+      <c r="E13" s="71"/>
+      <c r="F13" s="71"/>
+      <c r="G13" s="71"/>
+      <c r="H13" s="71"/>
+      <c r="I13" s="71"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="78"/>
+      <c r="L13" s="78"/>
+      <c r="M13" s="78"/>
+      <c r="N13" s="79" t="s">
         <v>43</v>
       </c>
-      <c r="O13" s="71"/>
-      <c r="P13" s="71"/>
-      <c r="Q13" s="72"/>
+      <c r="O13" s="80"/>
+      <c r="P13" s="80"/>
+      <c r="Q13" s="81"/>
     </row>
     <row r="14" spans="1:17" ht="27" customHeight="1">
-      <c r="A14" s="65"/>
-      <c r="B14" s="66"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="66"/>
-      <c r="H14" s="66"/>
-      <c r="I14" s="66"/>
-      <c r="J14" s="66"/>
-      <c r="K14" s="71" t="s">
+      <c r="A14" s="70"/>
+      <c r="B14" s="71"/>
+      <c r="C14" s="71"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="71"/>
+      <c r="F14" s="71"/>
+      <c r="G14" s="71"/>
+      <c r="H14" s="71"/>
+      <c r="I14" s="71"/>
+      <c r="J14" s="71"/>
+      <c r="K14" s="80" t="s">
         <v>34</v>
       </c>
-      <c r="L14" s="71"/>
-      <c r="M14" s="71"/>
-      <c r="N14" s="71"/>
-      <c r="O14" s="71"/>
-      <c r="P14" s="71"/>
-      <c r="Q14" s="72"/>
+      <c r="L14" s="80"/>
+      <c r="M14" s="80"/>
+      <c r="N14" s="80"/>
+      <c r="O14" s="80"/>
+      <c r="P14" s="80"/>
+      <c r="Q14" s="81"/>
     </row>
     <row r="15" spans="1:17" ht="255" customHeight="1">
-      <c r="A15" s="73"/>
-      <c r="B15" s="74"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
-      <c r="F15" s="74"/>
-      <c r="G15" s="74"/>
-      <c r="H15" s="74"/>
-      <c r="I15" s="74"/>
-      <c r="J15" s="74"/>
-      <c r="K15" s="75"/>
-      <c r="L15" s="75"/>
-      <c r="M15" s="75"/>
-      <c r="N15" s="75"/>
-      <c r="O15" s="75"/>
-      <c r="P15" s="75"/>
-      <c r="Q15" s="76"/>
+      <c r="A15" s="72"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
+      <c r="H15" s="73"/>
+      <c r="I15" s="73"/>
+      <c r="J15" s="73"/>
+      <c r="K15" s="82"/>
+      <c r="L15" s="82"/>
+      <c r="M15" s="82"/>
+      <c r="N15" s="82"/>
+      <c r="O15" s="82"/>
+      <c r="P15" s="82"/>
+      <c r="Q15" s="83"/>
     </row>
-    <row r="16" spans="1:17" s="79" customFormat="1" ht="15" customHeight="1">
-      <c r="A16" s="77"/>
-      <c r="B16" s="77"/>
-      <c r="C16" s="77"/>
-      <c r="D16" s="77"/>
-      <c r="E16" s="78"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="77"/>
-      <c r="H16" s="77"/>
-      <c r="I16" s="77"/>
-      <c r="J16" s="77"/>
-      <c r="K16" s="77"/>
-      <c r="L16" s="77"/>
-      <c r="M16" s="77"/>
-      <c r="N16" s="77"/>
-      <c r="O16" s="77"/>
-      <c r="P16" s="77"/>
-      <c r="Q16" s="77"/>
+    <row r="16" spans="1:17" s="20" customFormat="1" ht="15" customHeight="1">
+      <c r="A16" s="61"/>
+      <c r="B16" s="61"/>
+      <c r="C16" s="61"/>
+      <c r="D16" s="61"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="61"/>
+      <c r="G16" s="61"/>
+      <c r="H16" s="61"/>
+      <c r="I16" s="61"/>
+      <c r="J16" s="61"/>
+      <c r="K16" s="61"/>
+      <c r="L16" s="61"/>
+      <c r="M16" s="61"/>
+      <c r="N16" s="61"/>
+      <c r="O16" s="61"/>
+      <c r="P16" s="61"/>
+      <c r="Q16" s="61"/>
     </row>
-    <row r="17" spans="1:17" s="79" customFormat="1" ht="15" customHeight="1">
-      <c r="A17" s="77"/>
-      <c r="B17" s="77"/>
-      <c r="C17" s="77"/>
-      <c r="D17" s="77"/>
-      <c r="E17" s="78"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="77"/>
-      <c r="H17" s="77"/>
-      <c r="I17" s="77"/>
-      <c r="J17" s="77"/>
-      <c r="K17" s="77"/>
-      <c r="L17" s="77"/>
-      <c r="M17" s="77"/>
-      <c r="N17" s="77"/>
-      <c r="O17" s="77"/>
-      <c r="P17" s="77"/>
-      <c r="Q17" s="77"/>
+    <row r="17" spans="1:17" s="20" customFormat="1" ht="15" customHeight="1">
+      <c r="A17" s="61"/>
+      <c r="B17" s="61"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="61"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="61"/>
+      <c r="H17" s="61"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="61"/>
+      <c r="L17" s="61"/>
+      <c r="M17" s="61"/>
+      <c r="N17" s="61"/>
+      <c r="O17" s="61"/>
+      <c r="P17" s="61"/>
+      <c r="Q17" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="M2:M4"/>
-    <mergeCell ref="N2:N4"/>
-    <mergeCell ref="O2:O4"/>
-    <mergeCell ref="P2:P4"/>
-    <mergeCell ref="Q2:Q4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L2:L4"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="O6:O7"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:K2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A3:B4"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="F3:K4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="H6:H7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="A16:D17"/>
@@ -3581,9 +3576,40 @@
     <mergeCell ref="K14:Q15"/>
     <mergeCell ref="J6:J7"/>
     <mergeCell ref="K6:K7"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="F1:K2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="A3:B4"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F3:K4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="M2:M4"/>
+    <mergeCell ref="N2:N4"/>
+    <mergeCell ref="O2:O4"/>
+    <mergeCell ref="P2:P4"/>
+    <mergeCell ref="Q2:Q4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L2:L4"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="49" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="46" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>